<commit_message>
corrige el titulo no binario de fin_politica
Decia 'Punterr con unidad basica': un error de tipeo mio. Los otros doce
finales con variacion usan la terminacion en -e, asi que va 'Puntere'.
</commit_message>
<xml_diff>
--- a/eventos-pdf.xlsx
+++ b/eventos-pdf.xlsx
@@ -11493,12 +11493,16 @@
       <c r="J181" s="14" t="s">
         <v>706</v>
       </c>
-      <c r="K181" s="16"/>
+      <c r="K181" s="16" t="n">
+        <v>12</v>
+      </c>
       <c r="L181" s="16"/>
       <c r="M181" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="N181" s="16"/>
+      <c r="N181" s="16" t="n">
+        <v>12</v>
+      </c>
       <c r="O181" s="13" t="s">
         <v>187</v>
       </c>
@@ -15183,7 +15187,7 @@
       </c>
       <c r="G59" s="24" t="n">
         <f aca="false">SUMIF(Eventos!$A$2:$A$209,$A59,Eventos!$K$2:$K$209)</f>
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="H59" s="24" t="n">
         <f aca="false">SUMIF(Eventos!$A$2:$A$209,$A59,Eventos!$L$2:$L$209)</f>
@@ -15195,7 +15199,7 @@
       </c>
       <c r="J59" s="24" t="n">
         <f aca="false">SUMIF(Eventos!$A$2:$A$209,$A59,Eventos!$N$2:$N$209)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K59" s="23" t="n">
         <f aca="false">COUNTIFS(Eventos!$A$2:$A$209,$A59,Eventos!$Q$2:$Q$209,"&lt;&gt;")</f>
@@ -15586,7 +15590,7 @@
       </c>
       <c r="G69" s="26" t="n">
         <f aca="false">SUM(G2:G68)</f>
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="H69" s="26" t="n">
         <f aca="false">SUM(H2:H68)</f>
@@ -15598,7 +15602,7 @@
       </c>
       <c r="J69" s="26" t="n">
         <f aca="false">SUM(J2:J68)</f>
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="K69" s="25" t="n">
         <f aca="false">SUM(K2:K68)</f>

</xml_diff>

<commit_message>
placa compartible: el nombre va del mismo cuerpo que FSOQUER
Pasa de 8px a 13px y comparte linea de base (y+10, antes y+9): con el
mismo cuerpo, un pixel de diferencia se habria visto como un error.

Como el nombre lo escribe el jugador, se achica si no entra en lo que
queda entre FSOQUER y el margen derecho. Hoy no se activa nunca: quedan
329px libres, a 13px entran 25 caracteres y el campo del formulario
limita a 24. Es un seguro por si cambia alguno de los dos numeros.

El resto de la placa queda igual.
</commit_message>
<xml_diff>
--- a/eventos-pdf.xlsx
+++ b/eventos-pdf.xlsx
@@ -11493,9 +11493,7 @@
       <c r="J181" s="14" t="s">
         <v>706</v>
       </c>
-      <c r="K181" s="16" t="n">
-        <v>12</v>
-      </c>
+      <c r="K181" s="16"/>
       <c r="L181" s="16"/>
       <c r="M181" s="16" t="n">
         <v>12</v>
@@ -15187,7 +15185,7 @@
       </c>
       <c r="G59" s="24" t="n">
         <f aca="false">SUMIF(Eventos!$A$2:$A$209,$A59,Eventos!$K$2:$K$209)</f>
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="H59" s="24" t="n">
         <f aca="false">SUMIF(Eventos!$A$2:$A$209,$A59,Eventos!$L$2:$L$209)</f>
@@ -15590,7 +15588,7 @@
       </c>
       <c r="G69" s="26" t="n">
         <f aca="false">SUM(G2:G68)</f>
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="H69" s="26" t="n">
         <f aca="false">SUM(H2:H68)</f>

</xml_diff>